<commit_message>
Add 4 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (13):
- blocks/cards-product/cards-product.css
- blocks/columns-cta/columns-cta.css
- blocks/columns-intro/columns-intro.css
- blocks/columns-promo/columns-promo.css
- tools/importer/reports/contact-us.report.json
- tools/importer/reports/exercise-your-privacy-rights.report.json
- tools/importer/reports/free-samples.report.json
- tools/importer/reports/import-landing-page.report.xlsx
- tools/importer/reports/privacy.report.json
- tools/importer/reports/saves.report.json
- tools/importer/reports/stores.report.json
- tools/importer/reports/terms.report.json
- tools/importer/urls-utility.txt
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-landing-page.report.xlsx
+++ b/tools/importer/reports/import-landing-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="194">
   <si>
     <t>_reportFile</t>
   </si>
@@ -97,6 +97,51 @@
     <t>https://rouxbeauty.com/chocolate/</t>
   </si>
   <si>
+    <t>contact-us.report.json</t>
+  </si>
+  <si>
+    <t>contact-us</t>
+  </si>
+  <si>
+    <t>2026-05-20T16:25:13.908Z</t>
+  </si>
+  <si>
+    <t>Contact Us - RouxBeauty.com</t>
+  </si>
+  <si>
+    <t>https://rouxbeauty.com/contact-us/</t>
+  </si>
+  <si>
+    <t>exercise-your-privacy-rights.report.json</t>
+  </si>
+  <si>
+    <t>exercise-your-privacy-rights</t>
+  </si>
+  <si>
+    <t>2026-05-20T16:25:35.163Z</t>
+  </si>
+  <si>
+    <t>Exercise Your Privacy Rights - RouxBeauty.com</t>
+  </si>
+  <si>
+    <t>https://rouxbeauty.com/exercise-your-privacy-rights/</t>
+  </si>
+  <si>
+    <t>free-samples.report.json</t>
+  </si>
+  <si>
+    <t>free-samples</t>
+  </si>
+  <si>
+    <t>2026-05-20T16:25:49.522Z</t>
+  </si>
+  <si>
+    <t>Free Samples - RouxBeauty.com</t>
+  </si>
+  <si>
+    <t>https://rouxbeauty.com/free-samples/</t>
+  </si>
+  <si>
     <t>giving-thanks-to-you.report.json</t>
   </si>
   <si>
@@ -214,6 +259,21 @@
     <t>https://rouxbeauty.com/indulge-your-hair-with-rouxs-new-weightless-precious-oils-collection/</t>
   </si>
   <si>
+    <t>privacy.report.json</t>
+  </si>
+  <si>
+    <t>privacy</t>
+  </si>
+  <si>
+    <t>2026-05-20T16:25:20.889Z</t>
+  </si>
+  <si>
+    <t>Privacy - RouxBeauty.com</t>
+  </si>
+  <si>
+    <t>https://rouxbeauty.com/privacy/</t>
+  </si>
+  <si>
     <t>roux-tween-time-issuing-challenge-show-us-roots-america.report.json</t>
   </si>
   <si>
@@ -227,6 +287,51 @@
   </si>
   <si>
     <t>https://rouxbeauty.com/roux-tween-time-issuing-challenge-show-us-roots-america/</t>
+  </si>
+  <si>
+    <t>saves.report.json</t>
+  </si>
+  <si>
+    <t>saves</t>
+  </si>
+  <si>
+    <t>2026-05-20T16:25:42.055Z</t>
+  </si>
+  <si>
+    <t>Saves - RouxBeauty.com</t>
+  </si>
+  <si>
+    <t>https://rouxbeauty.com/saves/</t>
+  </si>
+  <si>
+    <t>stores.report.json</t>
+  </si>
+  <si>
+    <t>stores</t>
+  </si>
+  <si>
+    <t>2026-05-20T16:25:08.070Z</t>
+  </si>
+  <si>
+    <t>Stores - RouxBeauty.com</t>
+  </si>
+  <si>
+    <t>https://rouxbeauty.com/stores/</t>
+  </si>
+  <si>
+    <t>terms.report.json</t>
+  </si>
+  <si>
+    <t>terms</t>
+  </si>
+  <si>
+    <t>2026-05-20T16:25:27.640Z</t>
+  </si>
+  <si>
+    <t>Terms - RouxBeauty.com</t>
+  </si>
+  <si>
+    <t>https://rouxbeauty.com/terms/</t>
   </si>
   <si>
     <t>top-sellers.report.json</t>
@@ -876,7 +981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1046,62 +1151,62 @@
         <v>38</v>
       </c>
       <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
         <v>40</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>41</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>42</v>
-      </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
         <v>45</v>
       </c>
-      <c r="B8" t="s">
+      <c r="G8" t="s">
         <v>46</v>
       </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>47</v>
-      </c>
-      <c r="G8" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1110,76 +1215,76 @@
         <v>19</v>
       </c>
       <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
         <v>52</v>
-      </c>
-      <c r="G9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
         <v>56</v>
       </c>
-      <c r="C10" t="s">
+      <c r="F10" t="s">
         <v>57</v>
       </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="G10" t="s">
         <v>58</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H10" t="s">
         <v>59</v>
-      </c>
-      <c r="G10" t="s">
-        <v>60</v>
-      </c>
-      <c r="H10" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" t="s">
         <v>62</v>
       </c>
-      <c r="B11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="G11" t="s">
         <v>63</v>
       </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="H11" t="s">
         <v>64</v>
-      </c>
-      <c r="G11" t="s">
-        <v>65</v>
-      </c>
-      <c r="H11" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B12" t="s">
         <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -1188,50 +1293,50 @@
         <v>19</v>
       </c>
       <c r="F12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" t="s">
+        <v>68</v>
+      </c>
+      <c r="H12" t="s">
         <v>69</v>
-      </c>
-      <c r="G12" t="s">
-        <v>70</v>
-      </c>
-      <c r="H12" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
         <v>72</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
         <v>73</v>
       </c>
-      <c r="C13" t="s">
+      <c r="F13" t="s">
         <v>74</v>
       </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>75</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>76</v>
-      </c>
-      <c r="H13" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
         <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -1240,24 +1345,24 @@
         <v>19</v>
       </c>
       <c r="F14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" t="s">
         <v>80</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>81</v>
-      </c>
-      <c r="H14" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
         <v>17</v>
       </c>
       <c r="C15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -1266,10 +1371,10 @@
         <v>19</v>
       </c>
       <c r="F15" t="s">
+        <v>84</v>
+      </c>
+      <c r="G15" t="s">
         <v>85</v>
-      </c>
-      <c r="G15" t="s">
-        <v>60</v>
       </c>
       <c r="H15" t="s">
         <v>86</v>
@@ -1280,7 +1385,7 @@
         <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="C16" t="s">
         <v>88</v>
@@ -1289,7 +1394,7 @@
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="F16" t="s">
         <v>89</v>
@@ -1306,7 +1411,7 @@
         <v>92</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="C17" t="s">
         <v>93</v>
@@ -1315,7 +1420,7 @@
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="F17" t="s">
         <v>94</v>
@@ -1332,7 +1437,7 @@
         <v>97</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s">
         <v>98</v>
@@ -1341,7 +1446,7 @@
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="F18" t="s">
         <v>99</v>
@@ -1358,198 +1463,198 @@
         <v>102</v>
       </c>
       <c r="B19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" t="s">
         <v>103</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" t="s">
         <v>104</v>
       </c>
-      <c r="D19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="G19" t="s">
         <v>105</v>
       </c>
-      <c r="F19" t="s">
+      <c r="H19" t="s">
         <v>106</v>
-      </c>
-      <c r="G19" t="s">
-        <v>107</v>
-      </c>
-      <c r="H19" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" t="s">
+        <v>108</v>
+      </c>
+      <c r="C20" t="s">
         <v>109</v>
       </c>
-      <c r="B20" t="s">
-        <v>103</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>109</v>
+      </c>
+      <c r="F20" t="s">
         <v>110</v>
       </c>
-      <c r="D20" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" t="s">
-        <v>105</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>111</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>112</v>
-      </c>
-      <c r="H20" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>113</v>
+      </c>
+      <c r="B21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" t="s">
         <v>114</v>
       </c>
-      <c r="B21" t="s">
-        <v>103</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" t="s">
         <v>115</v>
       </c>
-      <c r="D21" t="s">
-        <v>11</v>
-      </c>
-      <c r="E21" t="s">
-        <v>105</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>116</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>117</v>
-      </c>
-      <c r="H21" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
         <v>119</v>
       </c>
-      <c r="B22" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" t="s">
         <v>120</v>
       </c>
-      <c r="D22" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" t="s">
-        <v>41</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
+        <v>75</v>
+      </c>
+      <c r="H22" t="s">
         <v>121</v>
-      </c>
-      <c r="G22" t="s">
-        <v>122</v>
-      </c>
-      <c r="H22" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>56</v>
+      </c>
+      <c r="F23" t="s">
         <v>124</v>
       </c>
-      <c r="B23" t="s">
-        <v>103</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="G23" t="s">
         <v>125</v>
       </c>
-      <c r="D23" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" t="s">
-        <v>105</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="H23" t="s">
         <v>126</v>
-      </c>
-      <c r="G23" t="s">
-        <v>127</v>
-      </c>
-      <c r="H23" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" t="s">
+        <v>128</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>56</v>
+      </c>
+      <c r="F24" t="s">
         <v>129</v>
       </c>
-      <c r="B24" t="s">
-        <v>103</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="G24" t="s">
         <v>130</v>
       </c>
-      <c r="D24" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" t="s">
-        <v>105</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="H24" t="s">
         <v>131</v>
-      </c>
-      <c r="G24" t="s">
-        <v>132</v>
-      </c>
-      <c r="H24" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" t="s">
+        <v>133</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>56</v>
+      </c>
+      <c r="F25" t="s">
         <v>134</v>
       </c>
-      <c r="B25" t="s">
-        <v>103</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="G25" t="s">
         <v>135</v>
       </c>
-      <c r="D25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" t="s">
-        <v>105</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="H25" t="s">
         <v>136</v>
-      </c>
-      <c r="G25" t="s">
-        <v>137</v>
-      </c>
-      <c r="H25" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>137</v>
+      </c>
+      <c r="B26" t="s">
+        <v>138</v>
+      </c>
+      <c r="C26" t="s">
         <v>139</v>
       </c>
-      <c r="B26" t="s">
-        <v>103</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
         <v>140</v>
-      </c>
-      <c r="D26" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" t="s">
-        <v>105</v>
       </c>
       <c r="F26" t="s">
         <v>141</v>
@@ -1566,7 +1671,7 @@
         <v>144</v>
       </c>
       <c r="B27" t="s">
-        <v>103</v>
+        <v>138</v>
       </c>
       <c r="C27" t="s">
         <v>145</v>
@@ -1575,7 +1680,7 @@
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="F27" t="s">
         <v>146</v>
@@ -1592,7 +1697,7 @@
         <v>149</v>
       </c>
       <c r="B28" t="s">
-        <v>103</v>
+        <v>138</v>
       </c>
       <c r="C28" t="s">
         <v>150</v>
@@ -1601,7 +1706,7 @@
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="F28" t="s">
         <v>151</v>
@@ -1618,7 +1723,7 @@
         <v>154</v>
       </c>
       <c r="B29" t="s">
-        <v>103</v>
+        <v>54</v>
       </c>
       <c r="C29" t="s">
         <v>155</v>
@@ -1627,7 +1732,7 @@
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>105</v>
+        <v>56</v>
       </c>
       <c r="F29" t="s">
         <v>156</v>
@@ -1637,6 +1742,188 @@
       </c>
       <c r="H29" t="s">
         <v>158</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>159</v>
+      </c>
+      <c r="B30" t="s">
+        <v>138</v>
+      </c>
+      <c r="C30" t="s">
+        <v>160</v>
+      </c>
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>140</v>
+      </c>
+      <c r="F30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G30" t="s">
+        <v>162</v>
+      </c>
+      <c r="H30" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>164</v>
+      </c>
+      <c r="B31" t="s">
+        <v>138</v>
+      </c>
+      <c r="C31" t="s">
+        <v>165</v>
+      </c>
+      <c r="D31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" t="s">
+        <v>140</v>
+      </c>
+      <c r="F31" t="s">
+        <v>166</v>
+      </c>
+      <c r="G31" t="s">
+        <v>167</v>
+      </c>
+      <c r="H31" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>169</v>
+      </c>
+      <c r="B32" t="s">
+        <v>138</v>
+      </c>
+      <c r="C32" t="s">
+        <v>170</v>
+      </c>
+      <c r="D32" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" t="s">
+        <v>140</v>
+      </c>
+      <c r="F32" t="s">
+        <v>171</v>
+      </c>
+      <c r="G32" t="s">
+        <v>172</v>
+      </c>
+      <c r="H32" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>174</v>
+      </c>
+      <c r="B33" t="s">
+        <v>138</v>
+      </c>
+      <c r="C33" t="s">
+        <v>175</v>
+      </c>
+      <c r="D33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" t="s">
+        <v>140</v>
+      </c>
+      <c r="F33" t="s">
+        <v>176</v>
+      </c>
+      <c r="G33" t="s">
+        <v>177</v>
+      </c>
+      <c r="H33" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>179</v>
+      </c>
+      <c r="B34" t="s">
+        <v>138</v>
+      </c>
+      <c r="C34" t="s">
+        <v>180</v>
+      </c>
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>140</v>
+      </c>
+      <c r="F34" t="s">
+        <v>181</v>
+      </c>
+      <c r="G34" t="s">
+        <v>182</v>
+      </c>
+      <c r="H34" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>184</v>
+      </c>
+      <c r="B35" t="s">
+        <v>138</v>
+      </c>
+      <c r="C35" t="s">
+        <v>185</v>
+      </c>
+      <c r="D35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
+        <v>140</v>
+      </c>
+      <c r="F35" t="s">
+        <v>186</v>
+      </c>
+      <c r="G35" t="s">
+        <v>187</v>
+      </c>
+      <c r="H35" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>189</v>
+      </c>
+      <c r="B36" t="s">
+        <v>138</v>
+      </c>
+      <c r="C36" t="s">
+        <v>190</v>
+      </c>
+      <c r="D36" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" t="s">
+        <v>140</v>
+      </c>
+      <c r="F36" t="s">
+        <v>191</v>
+      </c>
+      <c r="G36" t="s">
+        <v>192</v>
+      </c>
+      <c r="H36" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>